<commit_message>
Rename the Global lead persona to Nadia Hassan
Updates the sample data, Excel template and demo. Demo copies already
saved in a browser pick up the new name on their next load.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011uW1eDMqAYJJ1yh51RhwBP
</commit_message>
<xml_diff>
--- a/impact-tracker/sample-data/impact-tracker-template.xlsx
+++ b/impact-tracker/sample-data/impact-tracker-template.xlsx
@@ -8227,7 +8227,7 @@
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
@@ -8323,7 +8323,7 @@
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr">
@@ -8847,7 +8847,7 @@
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
@@ -8943,7 +8943,7 @@
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
@@ -9404,7 +9404,7 @@
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
       <c r="G4" s="10" t="inlineStr">
@@ -9454,7 +9454,7 @@
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -9500,7 +9500,7 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
@@ -9846,7 +9846,7 @@
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -14888,7 +14888,7 @@
       </c>
       <c r="E2" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor (Global lead)</t>
+          <t>Nadia Hassan (Global lead)</t>
         </is>
       </c>
       <c r="F2" s="10" t="inlineStr">
@@ -14954,7 +14954,7 @@
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor (Global lead)</t>
+          <t>Nadia Hassan (Global lead)</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
@@ -15129,7 +15129,7 @@
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor (Global lead) and GAPP</t>
+          <t>Nadia Hassan (Global lead) and GAPP</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr">
@@ -15216,7 +15216,7 @@
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
       <c r="E2" s="12" t="n">
@@ -16052,7 +16052,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
       <c r="B2" s="10" t="inlineStr">
@@ -16215,7 +16215,7 @@
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
       <c r="D2" s="11" t="n">
@@ -16275,7 +16275,7 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
       <c r="D5" s="11" t="n">
@@ -16428,7 +16428,7 @@
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
       <c r="E2" s="12" t="n">
@@ -16758,7 +16758,7 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
       <c r="E7" s="12" t="n">
@@ -22762,7 +22762,7 @@
       <c r="F2" s="3" t="n"/>
       <c r="G2" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -22820,7 +22820,7 @@
       <c r="F4" s="3" t="n"/>
       <c r="G4" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -22878,7 +22878,7 @@
       <c r="F6" s="3" t="n"/>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -22936,7 +22936,7 @@
       <c r="F8" s="3" t="n"/>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -22994,7 +22994,7 @@
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23052,7 +23052,7 @@
       <c r="F12" s="3" t="n"/>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23110,7 +23110,7 @@
       <c r="F14" s="3" t="n"/>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23168,7 +23168,7 @@
       <c r="F16" s="3" t="n"/>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23226,7 +23226,7 @@
       <c r="F18" s="3" t="n"/>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23284,7 +23284,7 @@
       <c r="F20" s="3" t="n"/>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23342,7 +23342,7 @@
       <c r="F22" s="3" t="n"/>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23400,7 +23400,7 @@
       <c r="F24" s="3" t="n"/>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23458,7 +23458,7 @@
       <c r="F26" s="3" t="n"/>
       <c r="G26" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23516,7 +23516,7 @@
       <c r="F28" s="3" t="n"/>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23574,7 +23574,7 @@
       <c r="F30" s="3" t="n"/>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23632,7 +23632,7 @@
       <c r="F32" s="3" t="n"/>
       <c r="G32" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23694,7 +23694,7 @@
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23752,7 +23752,7 @@
       <c r="F36" s="3" t="n"/>
       <c r="G36" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23810,7 +23810,7 @@
       <c r="F38" s="3" t="n"/>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23868,7 +23868,7 @@
       <c r="F40" s="3" t="n"/>
       <c r="G40" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23926,7 +23926,7 @@
       <c r="F42" s="3" t="n"/>
       <c r="G42" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -23984,7 +23984,7 @@
       <c r="F44" s="3" t="n"/>
       <c r="G44" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -24042,7 +24042,7 @@
       <c r="F46" s="3" t="n"/>
       <c r="G46" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>
@@ -24100,7 +24100,7 @@
       <c r="F48" s="3" t="n"/>
       <c r="G48" s="10" t="inlineStr">
         <is>
-          <t>Amira Okafor</t>
+          <t>Nadia Hassan</t>
         </is>
       </c>
     </row>

</xml_diff>